<commit_message>
feat: add secure account activation workflows
</commit_message>
<xml_diff>
--- a/docs/templates/modele_initialisation_plateforme_fyp.xlsx
+++ b/docs/templates/modele_initialisation_plateforme_fyp.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="1" r:id="R83a9c2582aa34355"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STUDENTS" sheetId="2" r:id="R75359ad1fa584cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ADMINISTRATORS" sheetId="3" r:id="R74f2da951e3f496d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COORDINATORS" sheetId="4" r:id="Ra9227190c5b2435e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUPERVISORS" sheetId="5" r:id="R1a54a4880fbe4b29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REPORT_EVALUATORS" sheetId="6" r:id="Re7e4e1a5cf064f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FACULTY_EVALUATORS" sheetId="7" r:id="Rc639571be0194914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDUSTRY_GUESTS" sheetId="8" r:id="Rd49eea0892ce43eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASES" sheetId="9" r:id="R16ba620c1d74480a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROJECT_ASSIGNMENTS" sheetId="10" r:id="R255e91e654ca4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="1" r:id="R0b0c4e2efc454b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STUDENTS" sheetId="2" r:id="Ra4a796c7120b4c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ADMINISTRATORS" sheetId="3" r:id="R275db08e1b334218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COORDINATORS" sheetId="4" r:id="Rc5f73a317a72449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUPERVISORS" sheetId="5" r:id="Re76bba599eca46ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REPORT_EVALUATORS" sheetId="6" r:id="R120d9029df574585"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FACULTY_EVALUATORS" sheetId="7" r:id="Ra019a9b5b06f4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDUSTRY_GUESTS" sheetId="8" r:id="R209cdcd4e2294b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASES" sheetId="9" r:id="Rcfa69ea128964a41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROJECT_ASSIGNMENTS" sheetId="10" r:id="R538eb04e74b741e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -638,7 +638,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>Replace each internal actor example with the official SQU identity. Do not add passwords; internal users authenticate through SQU SSO.</x:v>
+        <x:v>Replace each actor example with the official identity. Do not add passwords. Each user completes Sign up with the pre-registered email and a verification code sent by email.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32.25" customHeight="1">
@@ -646,7 +646,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
-        <x:v>For an Industry Guest, provide a future Access Expires At value and keep status PENDING_INVITATION. The platform sends a one-time activation link.</x:v>
+        <x:v>For an Industry Guest, provide a future Access Expires At value and use PENDING_ACTIVATION. The guest completes the same secure Sign up process.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32.25" customHeight="1">
@@ -686,7 +686,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>Upload the workbook in Excel Imports, run Preview, correct every error, then confirm the atomic import.</x:v>
+        <x:v>Upload the workbook in Excel Imports, run Preview, correct every error, then confirm the atomic import. To create an account active immediately, use Accounts and access after import.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -848,7 +848,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8b921f98c8a4baa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb306fab5f414d57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -928,7 +928,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc48024530e94467e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4061c9e29a04093"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -999,13 +999,18 @@
       <x:c r="G2" s="13" t="str"/>
       <x:c r="H2" s="30" t="str"/>
       <x:c r="I2" s="30" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"PENDING_ACTIVATION,ACTIVE,INACTIVE,SUSPENDED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb14fe8764d14e2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865ff094ba264c06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1076,13 +1081,18 @@
       <x:c r="G2" s="13" t="str"/>
       <x:c r="H2" s="30" t="str"/>
       <x:c r="I2" s="30" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"PENDING_ACTIVATION,ACTIVE,INACTIVE,SUSPENDED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radefc814626349db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068925014cde4922"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1153,7 +1163,7 @@
       <x:c r="G2" s="31" t="str"/>
       <x:c r="H2" s="28" t="str"/>
       <x:c r="I2" s="28" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="23.25" customHeight="1">
@@ -1178,13 +1188,18 @@
       <x:c r="G3" s="32" t="str"/>
       <x:c r="H3" s="29" t="str"/>
       <x:c r="I3" s="29" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"PENDING_ACTIVATION,ACTIVE,INACTIVE,SUSPENDED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c6db553ecc94b8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdcd344a08eb44c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1255,13 +1270,18 @@
       <x:c r="G2" s="13" t="str"/>
       <x:c r="H2" s="30" t="str"/>
       <x:c r="I2" s="30" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"PENDING_ACTIVATION,ACTIVE,INACTIVE,SUSPENDED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc72c323aa50944d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ffa7597e31a4406"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1332,13 +1352,18 @@
       <x:c r="G2" s="13" t="str"/>
       <x:c r="H2" s="30" t="str"/>
       <x:c r="I2" s="30" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"PENDING_ACTIVATION,ACTIVE,INACTIVE,SUSPENDED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1add5dd1ba7c41b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ef2ab0454bb4e7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1411,13 +1436,18 @@
         <x:v>2028-06-30T23:59</x:v>
       </x:c>
       <x:c r="I2" s="30" t="str">
-        <x:v>PENDING_INVITATION</x:v>
+        <x:v>PENDING_ACTIVATION</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"PENDING_ACTIVATION,ACTIVE,INACTIVE,SUSPENDED"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R033841fe23524c3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ad566af74f340cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1505,7 +1535,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R188f9b0532e94594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07aef37095ca4374"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>